<commit_message>
feat: implement interactive AGV vehicle simulation with animated routes and sound effects
Co-authored-by: jesusvanegas871 <287224091+jesusvanegas871@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/backend/data/inventario_maestro.xlsx
+++ b/backend/data/inventario_maestro.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PRODUCTOS A INCLUIR" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,599 +413,364 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>CODIGO</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Descripción</t>
+          <t>DESCRIPCIÓN</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Categoría ABC</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Ubicación</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Costo Unitario ($)</t>
+          <t>CATEGORIA</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REF-1001</t>
+          <t>SKU-1001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Empaque Metálico A1</t>
+          <t>Producto de Prueba 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Pasillo A - Estante 01</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F2" t="n">
-        <v>45.5</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REF-1002</t>
+          <t>SKU-1002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Motor Eléctrico 0.5HP</t>
+          <t>Producto de Prueba 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Pasillo A - Estante 02</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>350</v>
-      </c>
-      <c r="F3" t="n">
-        <v>280</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REF-1003</t>
+          <t>SKU-1003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rodamiento Industrial 6205</t>
+          <t>Producto de Prueba 3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Pasillo A - Estante 03</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F4" t="n">
-        <v>15.2</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REF-1004</t>
+          <t>SKU-1004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Válvula Hidráulica 3/4</t>
+          <t>Producto de Prueba 4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Pasillo A - Estante 04</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>420</v>
-      </c>
-      <c r="F5" t="n">
-        <v>110</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REF-1005</t>
+          <t>SKU-1005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sensor Optico Reflectivo</t>
+          <t>Producto de Prueba 5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Pasillo A - Estante 05</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>800</v>
-      </c>
-      <c r="F6" t="n">
-        <v>65</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REF-1006</t>
+          <t>SKU-1006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PLC Controlador M221</t>
+          <t>Producto de Prueba 6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Pasillo A - Estante 06</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>150</v>
-      </c>
-      <c r="F7" t="n">
-        <v>450</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>REF-1007</t>
+          <t>SKU-1007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Caja de Cartón Doble Corrugado</t>
+          <t>Producto de Prueba 7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Pasillo B - Estante 01</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2.1</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>REF-1008</t>
+          <t>SKU-1008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cinta Embalaje 48mm x 100m</t>
+          <t>Producto de Prueba 8</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Pasillo B - Estante 02</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>3200</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1.8</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>REF-1009</t>
+          <t>SKU-1009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Film Stretch 20 micras</t>
+          <t>Producto de Prueba 9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Pasillo B - Estante 03</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>1800</v>
-      </c>
-      <c r="F10" t="n">
-        <v>12.5</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>REF-1010</t>
+          <t>SKU-1010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Filtro Aceite Hidráulico</t>
+          <t>Producto de Prueba 10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Pasillo B - Estante 04</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>640</v>
-      </c>
-      <c r="F11" t="n">
-        <v>28</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>REF-1011</t>
+          <t>SKU-1011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Correa de Transmisión A-42</t>
+          <t>Producto de Prueba 11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Pasillo B - Estante 05</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>950</v>
-      </c>
-      <c r="F12" t="n">
-        <v>8.9</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>REF-1012</t>
+          <t>SKU-1012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Manguera Neumática 8mm</t>
+          <t>Producto de Prueba 12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Pasillo B - Estante 06</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>2100</v>
-      </c>
-      <c r="F13" t="n">
-        <v>4.3</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>REF-1013</t>
+          <t>SKU-1013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abrazadera Inoxidable 1 pulg</t>
+          <t>Producto de Prueba 13</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Pasillo C - Estante 01</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>8500</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.75</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REF-1014</t>
+          <t>SKU-1014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tornillo Grado 8 3/8x2</t>
+          <t>Producto de Prueba 14</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Pasillo C - Estante 02</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>12000</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.3</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>REF-1015</t>
+          <t>SKU-1015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tuerca de Seguridad M8</t>
+          <t>Producto de Prueba 15</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Pasillo C - Estante 03</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.15</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>REF-1016</t>
+          <t>SKU-1016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Arandela Plana 3/8</t>
+          <t>Producto de Prueba 16</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Pasillo C - Estante 04</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.08</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>REF-1017</t>
+          <t>SKU-1017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Conector Rápido Neumático</t>
+          <t>Producto de Prueba 17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Pasillo C - Estante 05</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>3100</v>
-      </c>
-      <c r="F18" t="n">
-        <v>2.4</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REF-1018</t>
+          <t>SKU-1018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Etiqueta Térmica 100x150mm</t>
+          <t>Producto de Prueba 18</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Pasillo C - Estante 06</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.05</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>REF-1019</t>
+          <t>SKU-1019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bomba de Agua Centrífuga</t>
+          <t>Producto de Prueba 19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Pasillo A - Estante 07</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>210</v>
-      </c>
-      <c r="F20" t="n">
-        <v>310</v>
+          <t>Categoría B</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>REF-1020</t>
+          <t>SKU-1020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Transformador 220V/24V</t>
+          <t>Producto de Prueba 20</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Pasillo B - Estante 07</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>430</v>
-      </c>
-      <c r="F21" t="n">
-        <v>55</v>
+          <t>Categoría A</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>